<commit_message>
fix test data & reguler master
</commit_message>
<xml_diff>
--- a/e2e/data/test-data-salary-deduction.xlsx
+++ b/e2e/data/test-data-salary-deduction.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:L6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,9 +430,12 @@
         <v>dplkEmployer</v>
       </c>
       <c r="J1" t="str">
+        <v>Potongan lain - lain</v>
+      </c>
+      <c r="K1" t="str">
         <v>totalExpected</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>totalEmployerExpected</v>
       </c>
     </row>
@@ -465,9 +468,12 @@
         <v>100000</v>
       </c>
       <c r="J2">
-        <v>25</v>
+        <v>100000</v>
       </c>
       <c r="K2">
+        <v>30</v>
+      </c>
+      <c r="L2">
         <v>5</v>
       </c>
     </row>
@@ -500,9 +506,12 @@
         <v>100000</v>
       </c>
       <c r="J3">
-        <v>35</v>
+        <v>100000</v>
       </c>
       <c r="K3">
+        <v>40</v>
+      </c>
+      <c r="L3">
         <v>5</v>
       </c>
     </row>
@@ -534,10 +543,13 @@
       <c r="I4">
         <v>100000</v>
       </c>
-      <c r="J4">
-        <v>35</v>
+      <c r="J4" t="str">
+        <v/>
       </c>
       <c r="K4">
+        <v>40</v>
+      </c>
+      <c r="L4">
         <v>5</v>
       </c>
     </row>
@@ -570,9 +582,12 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <v>25</v>
+        <v>100000</v>
       </c>
       <c r="K5">
+        <v>30</v>
+      </c>
+      <c r="L5">
         <v>0</v>
       </c>
     </row>
@@ -604,24 +619,26 @@
       <c r="I6">
         <v>0</v>
       </c>
-      <c r="J6">
-        <v>25</v>
+      <c r="J6" t="str">
+        <v/>
       </c>
       <c r="K6">
+        <v>30</v>
+      </c>
+      <c r="L6">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -655,15 +672,18 @@
         <v>employee13Seguranca</v>
       </c>
       <c r="K1" t="str">
+        <v>Potongan lain - lain</v>
+      </c>
+      <c r="L1" t="str">
         <v>totalExpected</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>employerSeguranca</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>employer13Seguranca</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>totalEmployerExpected</v>
       </c>
     </row>
@@ -699,15 +719,18 @@
         <v>50</v>
       </c>
       <c r="K2">
-        <v>1650</v>
+        <v>50</v>
       </c>
       <c r="L2">
+        <v>1700</v>
+      </c>
+      <c r="M2">
         <v>200</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>60</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>260</v>
       </c>
     </row>
@@ -743,15 +766,18 @@
         <v>50</v>
       </c>
       <c r="K3">
-        <v>2650</v>
+        <v>50</v>
       </c>
       <c r="L3">
+        <v>2700</v>
+      </c>
+      <c r="M3">
         <v>200</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>60</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>260</v>
       </c>
     </row>
@@ -786,16 +812,19 @@
       <c r="J4">
         <v>50</v>
       </c>
-      <c r="K4">
-        <v>2650</v>
+      <c r="K4" t="str">
+        <v/>
       </c>
       <c r="L4">
+        <v>2700</v>
+      </c>
+      <c r="M4">
         <v>200</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>60</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>260</v>
       </c>
     </row>
@@ -831,15 +860,18 @@
         <v>50</v>
       </c>
       <c r="K5">
-        <v>1650</v>
+        <v>50</v>
       </c>
       <c r="L5">
+        <v>1700</v>
+      </c>
+      <c r="M5">
         <v>200</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>60</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>260</v>
       </c>
     </row>
@@ -874,23 +906,25 @@
       <c r="J6">
         <v>50</v>
       </c>
-      <c r="K6">
-        <v>1650</v>
+      <c r="K6" t="str">
+        <v/>
       </c>
       <c r="L6">
+        <v>1700</v>
+      </c>
+      <c r="M6">
         <v>200</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>60</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>260</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
edit salary deduction test data
</commit_message>
<xml_diff>
--- a/e2e/data/test-data-salary-deduction.xlsx
+++ b/e2e/data/test-data-salary-deduction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Telkomcel\coding\test\e2e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72E3038-55E1-4E0C-A804-55FF9BBE6738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966E3B38-34F3-4C79-9B7D-F0CD629A474C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2100" windowWidth="23775" windowHeight="10140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homestaff" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="53">
   <si>
     <t>id</t>
   </si>
@@ -150,9 +150,6 @@
     <t>amount</t>
   </si>
   <si>
-    <t>2026-08</t>
-  </si>
-  <si>
     <t>Zakat Deduction</t>
   </si>
   <si>
@@ -169,9 +166,6 @@
   </si>
   <si>
     <t>TWP Deduction</t>
-  </si>
-  <si>
-    <t>2026-09</t>
   </si>
   <si>
     <t>IDP Deduction</t>
@@ -1266,22 +1260,22 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>44</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>45</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>46</v>
-      </c>
-      <c r="H2" t="s">
-        <v>47</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -1295,22 +1289,22 @@
         <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" t="s">
         <v>44</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>45</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>46</v>
-      </c>
-      <c r="H3" t="s">
-        <v>47</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1324,22 +1318,22 @@
         <v>13</v>
       </c>
       <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" t="s">
         <v>49</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>50</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>51</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>52</v>
-      </c>
-      <c r="G4" t="s">
-        <v>53</v>
-      </c>
-      <c r="H4" t="s">
-        <v>54</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1348,7 +1342,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I3 B4:I4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I1 B4 A3:B3 A2:B2 D2:I2 D3:I3 D4:I4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>